<commit_message>
chore: capture Realty Media workspace updates
</commit_message>
<xml_diff>
--- a/lead-list.xlsx
+++ b/lead-list.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Leads" sheetId="1" r:id="Ra39ba7694e4848c2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Leads" sheetId="1" r:id="Rbed19dfda0cf4f75"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -156,8 +156,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="LeadList" displayName="LeadList" ref="A1:K62" headerRowCount="1">
-  <x:autoFilter ref="A1:K62"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="LeadList" displayName="LeadList" ref="A1:K114" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A1:K114"/>
   <x:tableColumns count="11">
     <x:tableColumn id="1" name="Research Name of OWNER"/>
     <x:tableColumn id="2" name="County"/>
@@ -171,7 +171,7 @@
     <x:tableColumn id="10" name="Status"/>
     <x:tableColumn id="11" name="Source list"/>
   </x:tableColumns>
-  <x:tableStyleInfo name="TableStyleMedium2" showRowStripes="1"/>
+  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
 </file>
 
@@ -218,9 +218,9 @@
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Calibri"/>
-        <a:ea typeface="Calibri"/>
-        <a:cs typeface="Calibri"/>
+        <a:latin typeface="Calibri Light"/>
+        <a:ea typeface="Calibri Light"/>
+        <a:cs typeface="Calibri Light"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -372,7 +372,7 @@
   <x:cols>
     <x:col min="1" max="1" width="25.559999465942383" hidden="0" customWidth="1"/>
     <x:col min="2" max="2" width="9.4399995803833" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="21.110000610351562" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="23.329999923706055" hidden="0" customWidth="1"/>
     <x:col min="4" max="4" width="15" hidden="0" customWidth="1"/>
     <x:col min="5" max="5" width="27.219999313354492" hidden="0" customWidth="1"/>
     <x:col min="6" max="6" width="27.219999313354492" hidden="0" customWidth="1"/>
@@ -380,7 +380,7 @@
     <x:col min="8" max="8" width="27.219999313354492" hidden="0" customWidth="1"/>
     <x:col min="9" max="9" width="27.219999313354492" hidden="0" customWidth="1"/>
     <x:col min="10" max="10" width="11.670000076293945" hidden="0" customWidth="1"/>
-    <x:col min="11" max="11" width="14.4399995803833" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="16.670000076293945" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="24" customHeight="1">
@@ -440,7 +440,7 @@
       <x:c r="G2" s="7" t="str">
         <x:v>https://www.facebook.com/p/Charming-HOME-by-Feleacu-100068060672036/</x:v>
       </x:c>
-      <x:c r="H2" s="7" t="str"/>
+      <x:c r="H2" s="7"/>
       <x:c r="I2" s="7" t="str">
         <x:v>https://www.airbnb.com/rooms/26099368</x:v>
       </x:c>
@@ -467,11 +467,11 @@
       <x:c r="E3" s="7" t="str">
         <x:v>https://agropensiuneamaris.ro/</x:v>
       </x:c>
-      <x:c r="F3" s="7" t="str"/>
+      <x:c r="F3" s="7"/>
       <x:c r="G3" s="7" t="str">
         <x:v>https://www.facebook.com/pensiunemaris/?locale=ro_RO</x:v>
       </x:c>
-      <x:c r="H3" s="7" t="str"/>
+      <x:c r="H3" s="7"/>
       <x:c r="I3" s="7" t="str">
         <x:v>https://www.airbnb.com/rooms/26767830</x:v>
       </x:c>
@@ -495,10 +495,10 @@
       <x:c r="D4" s="7" t="str">
         <x:v>+40 757 767 594</x:v>
       </x:c>
-      <x:c r="E4" s="7" t="str"/>
-      <x:c r="F4" s="7" t="str"/>
-      <x:c r="G4" s="7" t="str"/>
-      <x:c r="H4" s="7" t="str"/>
+      <x:c r="E4" s="7"/>
+      <x:c r="F4" s="7"/>
+      <x:c r="G4" s="7"/>
+      <x:c r="H4" s="7"/>
       <x:c r="I4" s="7" t="str">
         <x:v>https://www.airbnb.com/rooms/1337012015906824814</x:v>
       </x:c>
@@ -522,10 +522,10 @@
       <x:c r="D5" s="7" t="str">
         <x:v>+40 749 094 933</x:v>
       </x:c>
-      <x:c r="E5" s="7" t="str"/>
-      <x:c r="F5" s="7" t="str"/>
-      <x:c r="G5" s="7" t="str"/>
-      <x:c r="H5" s="7" t="str"/>
+      <x:c r="E5" s="7"/>
+      <x:c r="F5" s="7"/>
+      <x:c r="G5" s="7"/>
+      <x:c r="H5" s="7"/>
       <x:c r="I5" s="7" t="str">
         <x:v>https://www.airbnb.com/rooms/1470264329893098656</x:v>
       </x:c>
@@ -549,10 +549,10 @@
       <x:c r="D6" s="7" t="str">
         <x:v>+40 758 573 583</x:v>
       </x:c>
-      <x:c r="E6" s="7" t="str"/>
-      <x:c r="F6" s="7" t="str"/>
-      <x:c r="G6" s="7" t="str"/>
-      <x:c r="H6" s="7" t="str"/>
+      <x:c r="E6" s="7"/>
+      <x:c r="F6" s="7"/>
+      <x:c r="G6" s="7"/>
+      <x:c r="H6" s="7"/>
       <x:c r="I6" s="7" t="str">
         <x:v>https://www.airbnb.com/rooms/1491882963947706361</x:v>
       </x:c>
@@ -579,9 +579,9 @@
       <x:c r="E7" s="7" t="str">
         <x:v>https://www.forestay.ro/cabana/peak-a-frame</x:v>
       </x:c>
-      <x:c r="F7" s="7" t="str"/>
-      <x:c r="G7" s="7" t="str"/>
-      <x:c r="H7" s="7" t="str"/>
+      <x:c r="F7" s="7"/>
+      <x:c r="G7" s="7"/>
+      <x:c r="H7" s="7"/>
       <x:c r="I7" s="7" t="str">
         <x:v>https://www.airbnb.com/rooms/1635574756084662230</x:v>
       </x:c>
@@ -614,7 +614,7 @@
       <x:c r="G8" s="7" t="str">
         <x:v>https://www.facebook.com/pedealulmieilor.ro/</x:v>
       </x:c>
-      <x:c r="H8" s="7" t="str"/>
+      <x:c r="H8" s="7"/>
       <x:c r="I8" s="7" t="str">
         <x:v>https://www.airbnb.com/rooms/1313197969723648366</x:v>
       </x:c>
@@ -638,10 +638,10 @@
       <x:c r="D9" s="7" t="str">
         <x:v>+40 754 327 876</x:v>
       </x:c>
-      <x:c r="E9" s="7" t="str"/>
-      <x:c r="F9" s="7" t="str"/>
-      <x:c r="G9" s="7" t="str"/>
-      <x:c r="H9" s="7" t="str"/>
+      <x:c r="E9" s="7"/>
+      <x:c r="F9" s="7"/>
+      <x:c r="G9" s="7"/>
+      <x:c r="H9" s="7"/>
       <x:c r="I9" s="7" t="str">
         <x:v>https://www.airbnb.com/rooms/1441450270421997693</x:v>
       </x:c>
@@ -665,10 +665,10 @@
       <x:c r="D10" s="7" t="str">
         <x:v>+40 755 461 100</x:v>
       </x:c>
-      <x:c r="E10" s="7" t="str"/>
-      <x:c r="F10" s="7" t="str"/>
-      <x:c r="G10" s="7" t="str"/>
-      <x:c r="H10" s="7" t="str"/>
+      <x:c r="E10" s="7"/>
+      <x:c r="F10" s="7"/>
+      <x:c r="G10" s="7"/>
+      <x:c r="H10" s="7"/>
       <x:c r="I10" s="7" t="str">
         <x:v>https://www.airbnb.com/rooms/1469551737443550810</x:v>
       </x:c>
@@ -695,9 +695,9 @@
       <x:c r="E11" s="7" t="str">
         <x:v>https://greenwoodcabin.com/en/greenwood-cabin</x:v>
       </x:c>
-      <x:c r="F11" s="7" t="str"/>
-      <x:c r="G11" s="7" t="str"/>
-      <x:c r="H11" s="7" t="str"/>
+      <x:c r="F11" s="7"/>
+      <x:c r="G11" s="7"/>
+      <x:c r="H11" s="7"/>
       <x:c r="I11" s="7" t="str">
         <x:v>https://www.airbnb.com/rooms/1163181833121581973</x:v>
       </x:c>
@@ -756,12 +756,12 @@
       <x:c r="D13" s="7" t="str">
         <x:v>+40 758 573 583</x:v>
       </x:c>
-      <x:c r="E13" s="7" t="str"/>
+      <x:c r="E13" s="7"/>
       <x:c r="F13" s="7" t="str">
         <x:v>https://www.instagram.com/nordlandcabin/</x:v>
       </x:c>
-      <x:c r="G13" s="7" t="str"/>
-      <x:c r="H13" s="7" t="str"/>
+      <x:c r="G13" s="7"/>
+      <x:c r="H13" s="7"/>
       <x:c r="I13" s="7" t="str">
         <x:v>https://www.airbnb.com/rooms/54138769</x:v>
       </x:c>
@@ -785,10 +785,10 @@
       <x:c r="D14" s="7" t="str">
         <x:v>+40 747 402 834</x:v>
       </x:c>
-      <x:c r="E14" s="7" t="str"/>
-      <x:c r="F14" s="7" t="str"/>
-      <x:c r="G14" s="7" t="str"/>
-      <x:c r="H14" s="7" t="str"/>
+      <x:c r="E14" s="7"/>
+      <x:c r="F14" s="7"/>
+      <x:c r="G14" s="7"/>
+      <x:c r="H14" s="7"/>
       <x:c r="I14" s="7" t="str">
         <x:v>https://www.airbnb.com/rooms/1375233243684550472</x:v>
       </x:c>
@@ -815,9 +815,9 @@
       <x:c r="E15" s="7" t="str">
         <x:v>https://atvmaguriracatau.ro/</x:v>
       </x:c>
-      <x:c r="F15" s="7" t="str"/>
-      <x:c r="G15" s="7" t="str"/>
-      <x:c r="H15" s="7" t="str"/>
+      <x:c r="F15" s="7"/>
+      <x:c r="G15" s="7"/>
+      <x:c r="H15" s="7"/>
       <x:c r="I15" s="7" t="str">
         <x:v>https://www.airbnb.com/rooms/1617412514246752822</x:v>
       </x:c>
@@ -841,10 +841,10 @@
       <x:c r="D16" s="7" t="str">
         <x:v>+40 740 729 051</x:v>
       </x:c>
-      <x:c r="E16" s="7" t="str"/>
-      <x:c r="F16" s="7" t="str"/>
-      <x:c r="G16" s="7" t="str"/>
-      <x:c r="H16" s="7" t="str"/>
+      <x:c r="E16" s="7"/>
+      <x:c r="F16" s="7"/>
+      <x:c r="G16" s="7"/>
+      <x:c r="H16" s="7"/>
       <x:c r="I16" s="7" t="str">
         <x:v>https://www.airbnb.com/rooms/585132500522176866</x:v>
       </x:c>
@@ -868,10 +868,10 @@
       <x:c r="D17" s="7" t="str">
         <x:v>+40 740 545 118</x:v>
       </x:c>
-      <x:c r="E17" s="7" t="str"/>
-      <x:c r="F17" s="7" t="str"/>
-      <x:c r="G17" s="7" t="str"/>
-      <x:c r="H17" s="7" t="str"/>
+      <x:c r="E17" s="7"/>
+      <x:c r="F17" s="7"/>
+      <x:c r="G17" s="7"/>
+      <x:c r="H17" s="7"/>
       <x:c r="I17" s="7" t="str">
         <x:v>https://www.airbnb.com/rooms/1643628598887992436</x:v>
       </x:c>
@@ -895,10 +895,10 @@
       <x:c r="D18" s="7" t="str">
         <x:v>+40 752 402 492</x:v>
       </x:c>
-      <x:c r="E18" s="7" t="str"/>
-      <x:c r="F18" s="7" t="str"/>
-      <x:c r="G18" s="7" t="str"/>
-      <x:c r="H18" s="7" t="str"/>
+      <x:c r="E18" s="7"/>
+      <x:c r="F18" s="7"/>
+      <x:c r="G18" s="7"/>
+      <x:c r="H18" s="7"/>
       <x:c r="I18" s="7" t="str">
         <x:v>https://www.airbnb.com/rooms/1425003008818298329</x:v>
       </x:c>
@@ -925,9 +925,9 @@
       <x:c r="E19" s="7" t="str">
         <x:v>https://arizonaranch.ro/</x:v>
       </x:c>
-      <x:c r="F19" s="7" t="str"/>
-      <x:c r="G19" s="7" t="str"/>
-      <x:c r="H19" s="7" t="str"/>
+      <x:c r="F19" s="7"/>
+      <x:c r="G19" s="7"/>
+      <x:c r="H19" s="7"/>
       <x:c r="I19" s="7" t="str">
         <x:v>https://www.airbnb.com/rooms/1241930004124203372</x:v>
       </x:c>
@@ -951,10 +951,10 @@
       <x:c r="D20" s="7" t="str">
         <x:v>+40 722 404 065</x:v>
       </x:c>
-      <x:c r="E20" s="7" t="str"/>
-      <x:c r="F20" s="7" t="str"/>
-      <x:c r="G20" s="7" t="str"/>
-      <x:c r="H20" s="7" t="str"/>
+      <x:c r="E20" s="7"/>
+      <x:c r="F20" s="7"/>
+      <x:c r="G20" s="7"/>
+      <x:c r="H20" s="7"/>
       <x:c r="I20" s="7" t="str">
         <x:v>https://www.airbnb.com/rooms/753320988710723911</x:v>
       </x:c>
@@ -978,10 +978,10 @@
       <x:c r="D21" s="7" t="str">
         <x:v>+40 741 213 380</x:v>
       </x:c>
-      <x:c r="E21" s="7" t="str"/>
-      <x:c r="F21" s="7" t="str"/>
-      <x:c r="G21" s="7" t="str"/>
-      <x:c r="H21" s="7" t="str"/>
+      <x:c r="E21" s="7"/>
+      <x:c r="F21" s="7"/>
+      <x:c r="G21" s="7"/>
+      <x:c r="H21" s="7"/>
       <x:c r="I21" s="7" t="str">
         <x:v>https://www.airbnb.com/rooms/1179821885707592528</x:v>
       </x:c>
@@ -1005,10 +1005,10 @@
       <x:c r="D22" s="7" t="str">
         <x:v>+40 771 655 828</x:v>
       </x:c>
-      <x:c r="E22" s="7" t="str"/>
-      <x:c r="F22" s="7" t="str"/>
-      <x:c r="G22" s="7" t="str"/>
-      <x:c r="H22" s="7" t="str"/>
+      <x:c r="E22" s="7"/>
+      <x:c r="F22" s="7"/>
+      <x:c r="G22" s="7"/>
+      <x:c r="H22" s="7"/>
       <x:c r="I22" s="7" t="str">
         <x:v>https://www.airbnb.com/rooms/1094792510594885861</x:v>
       </x:c>
@@ -1035,9 +1035,9 @@
       <x:c r="E23" s="7" t="str">
         <x:v>https://cabana-refugio.ro/</x:v>
       </x:c>
-      <x:c r="F23" s="7" t="str"/>
-      <x:c r="G23" s="7" t="str"/>
-      <x:c r="H23" s="7" t="str"/>
+      <x:c r="F23" s="7"/>
+      <x:c r="G23" s="7"/>
+      <x:c r="H23" s="7"/>
       <x:c r="I23" s="7" t="str">
         <x:v>https://www.airbnb.com/rooms/1133420905703577887</x:v>
       </x:c>
@@ -1061,10 +1061,10 @@
       <x:c r="D24" s="7" t="str">
         <x:v>+40 752 025 736</x:v>
       </x:c>
-      <x:c r="E24" s="7" t="str"/>
-      <x:c r="F24" s="7" t="str"/>
-      <x:c r="G24" s="7" t="str"/>
-      <x:c r="H24" s="7" t="str"/>
+      <x:c r="E24" s="7"/>
+      <x:c r="F24" s="7"/>
+      <x:c r="G24" s="7"/>
+      <x:c r="H24" s="7"/>
       <x:c r="I24" s="7" t="str">
         <x:v>https://www.airbnb.com/rooms/1086081028880930834</x:v>
       </x:c>
@@ -1088,10 +1088,10 @@
       <x:c r="D25" s="7" t="str">
         <x:v>+40 745 092 221</x:v>
       </x:c>
-      <x:c r="E25" s="7" t="str"/>
-      <x:c r="F25" s="7" t="str"/>
-      <x:c r="G25" s="7" t="str"/>
-      <x:c r="H25" s="7" t="str"/>
+      <x:c r="E25" s="7"/>
+      <x:c r="F25" s="7"/>
+      <x:c r="G25" s="7"/>
+      <x:c r="H25" s="7"/>
       <x:c r="I25" s="7" t="str">
         <x:v>https://www.airbnb.com/rooms/1283196307118483717</x:v>
       </x:c>
@@ -1115,10 +1115,10 @@
       <x:c r="D26" s="7" t="str">
         <x:v>+40 787 829 118</x:v>
       </x:c>
-      <x:c r="E26" s="7" t="str"/>
-      <x:c r="F26" s="7" t="str"/>
-      <x:c r="G26" s="7" t="str"/>
-      <x:c r="H26" s="7" t="str"/>
+      <x:c r="E26" s="7"/>
+      <x:c r="F26" s="7"/>
+      <x:c r="G26" s="7"/>
+      <x:c r="H26" s="7"/>
       <x:c r="I26" s="7" t="str">
         <x:v>https://www.airbnb.com/rooms/1603046487545912199</x:v>
       </x:c>
@@ -1145,9 +1145,9 @@
       <x:c r="E27" s="7" t="str">
         <x:v>https://cabanagoldensunset.ro/</x:v>
       </x:c>
-      <x:c r="F27" s="7" t="str"/>
-      <x:c r="G27" s="7" t="str"/>
-      <x:c r="H27" s="7" t="str"/>
+      <x:c r="F27" s="7"/>
+      <x:c r="G27" s="7"/>
+      <x:c r="H27" s="7"/>
       <x:c r="I27" s="7" t="str">
         <x:v>https://www.airbnb.com/rooms/1479678790365105081</x:v>
       </x:c>
@@ -1174,9 +1174,9 @@
       <x:c r="E28" s="7" t="str">
         <x:v>https://agropensiunea-mara.ro/</x:v>
       </x:c>
-      <x:c r="F28" s="7" t="str"/>
-      <x:c r="G28" s="7" t="str"/>
-      <x:c r="H28" s="7" t="str"/>
+      <x:c r="F28" s="7"/>
+      <x:c r="G28" s="7"/>
+      <x:c r="H28" s="7"/>
       <x:c r="I28" s="7" t="str">
         <x:v>https://www.airbnb.com/rooms/31870221</x:v>
       </x:c>
@@ -1200,10 +1200,10 @@
       <x:c r="D29" s="7" t="str">
         <x:v>+40 745 301 315</x:v>
       </x:c>
-      <x:c r="E29" s="7" t="str"/>
-      <x:c r="F29" s="7" t="str"/>
-      <x:c r="G29" s="7" t="str"/>
-      <x:c r="H29" s="7" t="str"/>
+      <x:c r="E29" s="7"/>
+      <x:c r="F29" s="7"/>
+      <x:c r="G29" s="7"/>
+      <x:c r="H29" s="7"/>
       <x:c r="I29" s="7" t="str">
         <x:v>https://www.airbnb.com/rooms/1321880941013349237</x:v>
       </x:c>
@@ -1230,9 +1230,9 @@
       <x:c r="E30" s="7" t="str">
         <x:v>https://monterosso.ro/</x:v>
       </x:c>
-      <x:c r="F30" s="7" t="str"/>
-      <x:c r="G30" s="7" t="str"/>
-      <x:c r="H30" s="7" t="str"/>
+      <x:c r="F30" s="7"/>
+      <x:c r="G30" s="7"/>
+      <x:c r="H30" s="7"/>
       <x:c r="I30" s="7" t="str">
         <x:v>https://www.airbnb.com/rooms/1505146237956562399</x:v>
       </x:c>
@@ -1259,9 +1259,9 @@
       <x:c r="E31" s="7" t="str">
         <x:v>https://nordikcabin.com/</x:v>
       </x:c>
-      <x:c r="F31" s="7" t="str"/>
-      <x:c r="G31" s="7" t="str"/>
-      <x:c r="H31" s="7" t="str"/>
+      <x:c r="F31" s="7"/>
+      <x:c r="G31" s="7"/>
+      <x:c r="H31" s="7"/>
       <x:c r="I31" s="7" t="str">
         <x:v>https://www.airbnb.com/rooms/1354807028958833716</x:v>
       </x:c>
@@ -1285,10 +1285,10 @@
       <x:c r="D32" s="7" t="str">
         <x:v>+40 745 032 285</x:v>
       </x:c>
-      <x:c r="E32" s="7" t="str"/>
-      <x:c r="F32" s="7" t="str"/>
-      <x:c r="G32" s="7" t="str"/>
-      <x:c r="H32" s="7" t="str"/>
+      <x:c r="E32" s="7"/>
+      <x:c r="F32" s="7"/>
+      <x:c r="G32" s="7"/>
+      <x:c r="H32" s="7"/>
       <x:c r="I32" s="7" t="str">
         <x:v>https://www.airbnb.com/rooms/1063162218344939189</x:v>
       </x:c>
@@ -1315,9 +1315,9 @@
       <x:c r="E33" s="7" t="str">
         <x:v>https://theviewmarisel.com/</x:v>
       </x:c>
-      <x:c r="F33" s="7" t="str"/>
-      <x:c r="G33" s="7" t="str"/>
-      <x:c r="H33" s="7" t="str"/>
+      <x:c r="F33" s="7"/>
+      <x:c r="G33" s="7"/>
+      <x:c r="H33" s="7"/>
       <x:c r="I33" s="7" t="str">
         <x:v>https://www.airbnb.com/rooms/1326939099856333219</x:v>
       </x:c>
@@ -1344,9 +1344,9 @@
       <x:c r="E34" s="7" t="str">
         <x:v>https://thenestcabin.com/</x:v>
       </x:c>
-      <x:c r="F34" s="7" t="str"/>
-      <x:c r="G34" s="7" t="str"/>
-      <x:c r="H34" s="7" t="str"/>
+      <x:c r="F34" s="7"/>
+      <x:c r="G34" s="7"/>
+      <x:c r="H34" s="7"/>
       <x:c r="I34" s="7" t="str">
         <x:v>https://www.airbnb.com/rooms/1315291316782237714</x:v>
       </x:c>
@@ -1370,10 +1370,10 @@
       <x:c r="D35" s="7" t="str">
         <x:v>+40 740 185 730</x:v>
       </x:c>
-      <x:c r="E35" s="7" t="str"/>
-      <x:c r="F35" s="7" t="str"/>
-      <x:c r="G35" s="7" t="str"/>
-      <x:c r="H35" s="7" t="str"/>
+      <x:c r="E35" s="7"/>
+      <x:c r="F35" s="7"/>
+      <x:c r="G35" s="7"/>
+      <x:c r="H35" s="7"/>
       <x:c r="I35" s="7" t="str">
         <x:v>https://www.airbnb.com/rooms/1197049207881229146</x:v>
       </x:c>
@@ -1397,10 +1397,10 @@
       <x:c r="D36" s="7" t="str">
         <x:v>+40 755 096 699</x:v>
       </x:c>
-      <x:c r="E36" s="7" t="str"/>
-      <x:c r="F36" s="7" t="str"/>
-      <x:c r="G36" s="7" t="str"/>
-      <x:c r="H36" s="7" t="str"/>
+      <x:c r="E36" s="7"/>
+      <x:c r="F36" s="7"/>
+      <x:c r="G36" s="7"/>
+      <x:c r="H36" s="7"/>
       <x:c r="I36" s="7" t="str">
         <x:v>https://www.airbnb.com/rooms/764951439111893168</x:v>
       </x:c>
@@ -1424,10 +1424,10 @@
       <x:c r="D37" s="7" t="str">
         <x:v>+40 733 871 941</x:v>
       </x:c>
-      <x:c r="E37" s="7" t="str"/>
-      <x:c r="F37" s="7" t="str"/>
-      <x:c r="G37" s="7" t="str"/>
-      <x:c r="H37" s="7" t="str"/>
+      <x:c r="E37" s="7"/>
+      <x:c r="F37" s="7"/>
+      <x:c r="G37" s="7"/>
+      <x:c r="H37" s="7"/>
       <x:c r="I37" s="7" t="str">
         <x:v>https://www.airbnb.com/rooms/1511092554926308882</x:v>
       </x:c>
@@ -1451,10 +1451,10 @@
       <x:c r="D38" s="7" t="str">
         <x:v>+40 760 294 786</x:v>
       </x:c>
-      <x:c r="E38" s="7" t="str"/>
-      <x:c r="F38" s="7" t="str"/>
-      <x:c r="G38" s="7" t="str"/>
-      <x:c r="H38" s="7" t="str"/>
+      <x:c r="E38" s="7"/>
+      <x:c r="F38" s="7"/>
+      <x:c r="G38" s="7"/>
+      <x:c r="H38" s="7"/>
       <x:c r="I38" s="7" t="str">
         <x:v>https://www.airbnb.com/rooms/1019387524748730856</x:v>
       </x:c>
@@ -1478,10 +1478,10 @@
       <x:c r="D39" s="7" t="str">
         <x:v>+40 723 692 027</x:v>
       </x:c>
-      <x:c r="E39" s="7" t="str"/>
-      <x:c r="F39" s="7" t="str"/>
-      <x:c r="G39" s="7" t="str"/>
-      <x:c r="H39" s="7" t="str"/>
+      <x:c r="E39" s="7"/>
+      <x:c r="F39" s="7"/>
+      <x:c r="G39" s="7"/>
+      <x:c r="H39" s="7"/>
       <x:c r="I39" s="7" t="str">
         <x:v>https://www.airbnb.com/rooms/962753684964916516</x:v>
       </x:c>
@@ -1505,10 +1505,10 @@
       <x:c r="D40" s="7" t="str">
         <x:v>+40 749 200 087</x:v>
       </x:c>
-      <x:c r="E40" s="7" t="str"/>
-      <x:c r="F40" s="7" t="str"/>
-      <x:c r="G40" s="7" t="str"/>
-      <x:c r="H40" s="7" t="str"/>
+      <x:c r="E40" s="7"/>
+      <x:c r="F40" s="7"/>
+      <x:c r="G40" s="7"/>
+      <x:c r="H40" s="7"/>
       <x:c r="I40" s="7" t="str">
         <x:v>https://www.airbnb.com/rooms/973769914274124440</x:v>
       </x:c>
@@ -1532,10 +1532,10 @@
       <x:c r="D41" s="7" t="str">
         <x:v>+40 746 267 634</x:v>
       </x:c>
-      <x:c r="E41" s="7" t="str"/>
-      <x:c r="F41" s="7" t="str"/>
-      <x:c r="G41" s="7" t="str"/>
-      <x:c r="H41" s="7" t="str"/>
+      <x:c r="E41" s="7"/>
+      <x:c r="F41" s="7"/>
+      <x:c r="G41" s="7"/>
+      <x:c r="H41" s="7"/>
       <x:c r="I41" s="7" t="str">
         <x:v>https://www.airbnb.com/rooms/924462515882386562</x:v>
       </x:c>
@@ -1559,10 +1559,10 @@
       <x:c r="D42" s="7" t="str">
         <x:v>+40 743 185 302</x:v>
       </x:c>
-      <x:c r="E42" s="7" t="str"/>
-      <x:c r="F42" s="7" t="str"/>
-      <x:c r="G42" s="7" t="str"/>
-      <x:c r="H42" s="7" t="str"/>
+      <x:c r="E42" s="7"/>
+      <x:c r="F42" s="7"/>
+      <x:c r="G42" s="7"/>
+      <x:c r="H42" s="7"/>
       <x:c r="I42" s="7" t="str">
         <x:v>https://www.airbnb.com/rooms/760138116186242116</x:v>
       </x:c>
@@ -1589,9 +1589,9 @@
       <x:c r="E43" s="7" t="str">
         <x:v>https://pensiunea-caesarshouse.ro/</x:v>
       </x:c>
-      <x:c r="F43" s="7" t="str"/>
-      <x:c r="G43" s="7" t="str"/>
-      <x:c r="H43" s="7" t="str"/>
+      <x:c r="F43" s="7"/>
+      <x:c r="G43" s="7"/>
+      <x:c r="H43" s="7"/>
       <x:c r="I43" s="7" t="str">
         <x:v>https://www.airbnb.com/rooms/1679055975215304856</x:v>
       </x:c>
@@ -1615,10 +1615,10 @@
       <x:c r="D44" s="7" t="str">
         <x:v>+40 757 011 128</x:v>
       </x:c>
-      <x:c r="E44" s="7" t="str"/>
-      <x:c r="F44" s="7" t="str"/>
-      <x:c r="G44" s="7" t="str"/>
-      <x:c r="H44" s="7" t="str"/>
+      <x:c r="E44" s="7"/>
+      <x:c r="F44" s="7"/>
+      <x:c r="G44" s="7"/>
+      <x:c r="H44" s="7"/>
       <x:c r="I44" s="7" t="str">
         <x:v>https://www.airbnb.com/rooms/41386599</x:v>
       </x:c>
@@ -1642,10 +1642,10 @@
       <x:c r="D45" s="7" t="str">
         <x:v>+40 749 315 604</x:v>
       </x:c>
-      <x:c r="E45" s="7" t="str"/>
-      <x:c r="F45" s="7" t="str"/>
-      <x:c r="G45" s="7" t="str"/>
-      <x:c r="H45" s="7" t="str"/>
+      <x:c r="E45" s="7"/>
+      <x:c r="F45" s="7"/>
+      <x:c r="G45" s="7"/>
+      <x:c r="H45" s="7"/>
       <x:c r="I45" s="7" t="str">
         <x:v>https://www.airbnb.com/rooms/777550357867234122</x:v>
       </x:c>
@@ -1669,10 +1669,10 @@
       <x:c r="D46" s="7" t="str">
         <x:v>+40 740 146 596</x:v>
       </x:c>
-      <x:c r="E46" s="7" t="str"/>
-      <x:c r="F46" s="7" t="str"/>
-      <x:c r="G46" s="7" t="str"/>
-      <x:c r="H46" s="7" t="str"/>
+      <x:c r="E46" s="7"/>
+      <x:c r="F46" s="7"/>
+      <x:c r="G46" s="7"/>
+      <x:c r="H46" s="7"/>
       <x:c r="I46" s="7" t="str">
         <x:v>https://www.airbnb.com/rooms/1410306856300432538</x:v>
       </x:c>
@@ -1696,10 +1696,10 @@
       <x:c r="D47" s="7" t="str">
         <x:v>+40 748 196 905</x:v>
       </x:c>
-      <x:c r="E47" s="7" t="str"/>
-      <x:c r="F47" s="7" t="str"/>
-      <x:c r="G47" s="7" t="str"/>
-      <x:c r="H47" s="7" t="str"/>
+      <x:c r="E47" s="7"/>
+      <x:c r="F47" s="7"/>
+      <x:c r="G47" s="7"/>
+      <x:c r="H47" s="7"/>
       <x:c r="I47" s="7" t="str">
         <x:v>https://www.airbnb.com/rooms/606868356836278107</x:v>
       </x:c>
@@ -1723,10 +1723,10 @@
       <x:c r="D48" s="7" t="str">
         <x:v>+40 728 830 373</x:v>
       </x:c>
-      <x:c r="E48" s="7" t="str"/>
-      <x:c r="F48" s="7" t="str"/>
-      <x:c r="G48" s="7" t="str"/>
-      <x:c r="H48" s="7" t="str"/>
+      <x:c r="E48" s="7"/>
+      <x:c r="F48" s="7"/>
+      <x:c r="G48" s="7"/>
+      <x:c r="H48" s="7"/>
       <x:c r="I48" s="7" t="str">
         <x:v>https://www.airbnb.com/rooms/1205035395571461396</x:v>
       </x:c>
@@ -1750,10 +1750,10 @@
       <x:c r="D49" s="7" t="str">
         <x:v>+40 733 117 686</x:v>
       </x:c>
-      <x:c r="E49" s="7" t="str"/>
-      <x:c r="F49" s="7" t="str"/>
-      <x:c r="G49" s="7" t="str"/>
-      <x:c r="H49" s="7" t="str"/>
+      <x:c r="E49" s="7"/>
+      <x:c r="F49" s="7"/>
+      <x:c r="G49" s="7"/>
+      <x:c r="H49" s="7"/>
       <x:c r="I49" s="7" t="str">
         <x:v>https://www.airbnb.com/rooms/557299790053916975</x:v>
       </x:c>
@@ -1780,11 +1780,11 @@
       <x:c r="E50" s="7" t="str">
         <x:v>https://pensiuneajunior.ro/</x:v>
       </x:c>
-      <x:c r="F50" s="7" t="str"/>
+      <x:c r="F50" s="7"/>
       <x:c r="G50" s="7" t="str">
         <x:v>https://www.facebook.com/pensiunejunior/</x:v>
       </x:c>
-      <x:c r="H50" s="7" t="str"/>
+      <x:c r="H50" s="7"/>
       <x:c r="I50" s="7" t="str">
         <x:v>https://pensiuneajunior.ro/</x:v>
       </x:c>
@@ -1811,9 +1811,9 @@
       <x:c r="E51" s="7" t="str">
         <x:v>https://www.pensiuneazbor.ro/</x:v>
       </x:c>
-      <x:c r="F51" s="7" t="str"/>
-      <x:c r="G51" s="7" t="str"/>
-      <x:c r="H51" s="7" t="str"/>
+      <x:c r="F51" s="7"/>
+      <x:c r="G51" s="7"/>
+      <x:c r="H51" s="7"/>
       <x:c r="I51" s="7" t="str">
         <x:v>https://www.pensiuneazbor.ro/</x:v>
       </x:c>
@@ -1840,9 +1840,9 @@
       <x:c r="E52" s="7" t="str">
         <x:v>https://www.vilasiago.ro/</x:v>
       </x:c>
-      <x:c r="F52" s="7" t="str"/>
-      <x:c r="G52" s="7" t="str"/>
-      <x:c r="H52" s="7" t="str"/>
+      <x:c r="F52" s="7"/>
+      <x:c r="G52" s="7"/>
+      <x:c r="H52" s="7"/>
       <x:c r="I52" s="7" t="str">
         <x:v>https://www.vilasiago.ro/</x:v>
       </x:c>
@@ -1869,9 +1869,9 @@
       <x:c r="E53" s="7" t="str">
         <x:v>https://pensiuneasada.ro/</x:v>
       </x:c>
-      <x:c r="F53" s="7" t="str"/>
-      <x:c r="G53" s="7" t="str"/>
-      <x:c r="H53" s="7" t="str"/>
+      <x:c r="F53" s="7"/>
+      <x:c r="G53" s="7"/>
+      <x:c r="H53" s="7"/>
       <x:c r="I53" s="7" t="str">
         <x:v>https://pensiuneasada.ro/contact/</x:v>
       </x:c>
@@ -1904,7 +1904,7 @@
       <x:c r="G54" s="7" t="str">
         <x:v>https://www.facebook.com/transylvaniavillabaisoara</x:v>
       </x:c>
-      <x:c r="H54" s="7" t="str"/>
+      <x:c r="H54" s="7"/>
       <x:c r="I54" s="7" t="str">
         <x:v>http://baisoara.transylvaniavilla.com</x:v>
       </x:c>
@@ -1931,11 +1931,11 @@
       <x:c r="E55" s="7" t="str">
         <x:v>https://lamesteceni.ro/</x:v>
       </x:c>
-      <x:c r="F55" s="7" t="str"/>
+      <x:c r="F55" s="7"/>
       <x:c r="G55" s="7" t="str">
         <x:v>https://www.facebook.com/PensiuneaLaMesteceni</x:v>
       </x:c>
-      <x:c r="H55" s="7" t="str"/>
+      <x:c r="H55" s="7"/>
       <x:c r="I55" s="7" t="str">
         <x:v>https://lamesteceni.ro/</x:v>
       </x:c>
@@ -1962,9 +1962,9 @@
       <x:c r="E56" s="7" t="str">
         <x:v>https://pensiuneacionca.ro/</x:v>
       </x:c>
-      <x:c r="F56" s="7" t="str"/>
-      <x:c r="G56" s="7" t="str"/>
-      <x:c r="H56" s="7" t="str"/>
+      <x:c r="F56" s="7"/>
+      <x:c r="G56" s="7"/>
+      <x:c r="H56" s="7"/>
       <x:c r="I56" s="7" t="str">
         <x:v>https://pensiuneacionca.ro/</x:v>
       </x:c>
@@ -1988,10 +1988,10 @@
       <x:c r="D57" s="7" t="str">
         <x:v>+40 728 182 032</x:v>
       </x:c>
-      <x:c r="E57" s="7" t="str"/>
-      <x:c r="F57" s="7" t="str"/>
-      <x:c r="G57" s="7" t="str"/>
-      <x:c r="H57" s="7" t="str"/>
+      <x:c r="E57" s="7"/>
+      <x:c r="F57" s="7"/>
+      <x:c r="G57" s="7"/>
+      <x:c r="H57" s="7"/>
       <x:c r="I57" s="7" t="str">
         <x:v>https://carta.ro/cazare-statiunea-muntele-baisorii/pensiunea-skiland/</x:v>
       </x:c>
@@ -2015,10 +2015,10 @@
       <x:c r="D58" s="7" t="str">
         <x:v>+40 741 946 460</x:v>
       </x:c>
-      <x:c r="E58" s="7" t="str"/>
-      <x:c r="F58" s="7" t="str"/>
-      <x:c r="G58" s="7" t="str"/>
-      <x:c r="H58" s="7" t="str"/>
+      <x:c r="E58" s="7"/>
+      <x:c r="F58" s="7"/>
+      <x:c r="G58" s="7"/>
+      <x:c r="H58" s="7"/>
       <x:c r="I58" s="7" t="str">
         <x:v>https://carta.ro/cazare-turda/pensiunea-edy/</x:v>
       </x:c>
@@ -2042,10 +2042,10 @@
       <x:c r="D59" s="7" t="str">
         <x:v>+40 747 936 523</x:v>
       </x:c>
-      <x:c r="E59" s="7" t="str"/>
-      <x:c r="F59" s="7" t="str"/>
-      <x:c r="G59" s="7" t="str"/>
-      <x:c r="H59" s="7" t="str"/>
+      <x:c r="E59" s="7"/>
+      <x:c r="F59" s="7"/>
+      <x:c r="G59" s="7"/>
+      <x:c r="H59" s="7"/>
       <x:c r="I59" s="7" t="str">
         <x:v>https://carta.ro/cazare-turda/pensiunea-perla-transilvaniei/</x:v>
       </x:c>
@@ -2069,10 +2069,10 @@
       <x:c r="D60" s="7" t="str">
         <x:v>+40 745 659 212</x:v>
       </x:c>
-      <x:c r="E60" s="7" t="str"/>
-      <x:c r="F60" s="7" t="str"/>
-      <x:c r="G60" s="7" t="str"/>
-      <x:c r="H60" s="7" t="str"/>
+      <x:c r="E60" s="7"/>
+      <x:c r="F60" s="7"/>
+      <x:c r="G60" s="7"/>
+      <x:c r="H60" s="7"/>
       <x:c r="I60" s="7" t="str">
         <x:v>https://carta.ro/cazare-turda/casa-alin/</x:v>
       </x:c>
@@ -2096,10 +2096,10 @@
       <x:c r="D61" s="7" t="str">
         <x:v>+40 745 775 178</x:v>
       </x:c>
-      <x:c r="E61" s="7" t="str"/>
-      <x:c r="F61" s="7" t="str"/>
-      <x:c r="G61" s="7" t="str"/>
-      <x:c r="H61" s="7" t="str"/>
+      <x:c r="E61" s="7"/>
+      <x:c r="F61" s="7"/>
+      <x:c r="G61" s="7"/>
+      <x:c r="H61" s="7"/>
       <x:c r="I61" s="7" t="str">
         <x:v>https://carta.ro/cazare-floresti/pensiunea-maria/</x:v>
       </x:c>
@@ -2111,46 +2111,1568 @@
       </x:c>
     </x:row>
     <x:row r="62" ht="31.5" customHeight="1">
-      <x:c r="A62" s="8" t="str">
+      <x:c r="A62" s="7" t="str">
         <x:v>Cabana LA IONEL</x:v>
       </x:c>
-      <x:c r="B62" s="8" t="str">
-        <x:v>Cluj</x:v>
-      </x:c>
-      <x:c r="C62" s="8" t="str">
+      <x:c r="B62" s="7" t="str">
+        <x:v>Cluj</x:v>
+      </x:c>
+      <x:c r="C62" s="7" t="str">
         <x:v>Măguri-Răcătău, jud. Cluj</x:v>
       </x:c>
-      <x:c r="D62" s="8" t="str">
+      <x:c r="D62" s="7" t="str">
         <x:v>+40 740 946 121</x:v>
       </x:c>
-      <x:c r="E62" s="8" t="str"/>
-      <x:c r="F62" s="8" t="str"/>
-      <x:c r="G62" s="8" t="str"/>
-      <x:c r="H62" s="8" t="str"/>
-      <x:c r="I62" s="8" t="str">
+      <x:c r="E62" s="7"/>
+      <x:c r="F62" s="7"/>
+      <x:c r="G62" s="7"/>
+      <x:c r="H62" s="7"/>
+      <x:c r="I62" s="7" t="str">
         <x:v>https://carta.ro/cazare-maguri-racatau/cabana-la-ionel/</x:v>
       </x:c>
-      <x:c r="J62" s="14" t="str">
-        <x:v>Pending</x:v>
-      </x:c>
-      <x:c r="K62" s="8" t="str">
+      <x:c r="J62" s="13" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="K62" s="7" t="str">
         <x:v>Măguri-Răcătău</x:v>
       </x:c>
     </x:row>
+    <x:row r="63" ht="31.5" customHeight="1">
+      <x:c r="A63" s="7" t="str">
+        <x:v>Elite City / Elite Grup</x:v>
+      </x:c>
+      <x:c r="B63" s="7" t="str">
+        <x:v>Cluj</x:v>
+      </x:c>
+      <x:c r="C63" s="7" t="str">
+        <x:v>Bulevardul Muncii / zona Fabricii, Cluj-Napoca</x:v>
+      </x:c>
+      <x:c r="D63" s="7" t="str">
+        <x:v>+40 740 711 200</x:v>
+      </x:c>
+      <x:c r="E63" s="7" t="str">
+        <x:v>https://www.elite.ro/</x:v>
+      </x:c>
+      <x:c r="F63" s="7" t="str">
+        <x:v>https://www.instagram.com/elitecitycluj/</x:v>
+      </x:c>
+      <x:c r="G63" s="7" t="str">
+        <x:v>https://www.facebook.com/elitecitycluj</x:v>
+      </x:c>
+      <x:c r="H63" s="7"/>
+      <x:c r="I63" s="7" t="str">
+        <x:v>https://www.elite.ro/elitecity/apartamente</x:v>
+      </x:c>
+      <x:c r="J63" s="13" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="K63" s="7" t="str">
+        <x:v>Dezvoltatori Cluj / Cluj-Napoca</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="64" ht="31.5" customHeight="1">
+      <x:c r="A64" s="7" t="str">
+        <x:v>Maurer Panoramic / Maurer Imobiliare</x:v>
+      </x:c>
+      <x:c r="B64" s="7" t="str">
+        <x:v>Cluj</x:v>
+      </x:c>
+      <x:c r="C64" s="7" t="str">
+        <x:v>Str. Lalelelor nr. 14, Cluj-Napoca</x:v>
+      </x:c>
+      <x:c r="D64" s="7" t="str">
+        <x:v>+40 784 441 111</x:v>
+      </x:c>
+      <x:c r="E64" s="7" t="str">
+        <x:v>https://www.maurerpanoramic.ro/</x:v>
+      </x:c>
+      <x:c r="F64" s="7" t="str">
+        <x:v>https://www.instagram.com/maurerpanoramic</x:v>
+      </x:c>
+      <x:c r="G64" s="7" t="str">
+        <x:v>https://www.facebook.com/pages/category/Apartment---Condo-Building/Maurer-Panoramic-737527903245924/</x:v>
+      </x:c>
+      <x:c r="H64" s="7"/>
+      <x:c r="I64" s="7" t="str">
+        <x:v>https://www.maurerpanoramic.ro/</x:v>
+      </x:c>
+      <x:c r="J64" s="13" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="K64" s="7" t="str">
+        <x:v>Dezvoltatori Cluj / Cluj-Napoca</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="65" ht="31.5" customHeight="1">
+      <x:c r="A65" s="7" t="str">
+        <x:v>Oxygen Residence</x:v>
+      </x:c>
+      <x:c r="B65" s="7" t="str">
+        <x:v>Cluj</x:v>
+      </x:c>
+      <x:c r="C65" s="7" t="str">
+        <x:v>Piața Abator 1, Cluj-Napoca</x:v>
+      </x:c>
+      <x:c r="D65" s="7" t="str">
+        <x:v>+40 734 335 104</x:v>
+      </x:c>
+      <x:c r="E65" s="7" t="str">
+        <x:v>https://oxygencluj.ro/</x:v>
+      </x:c>
+      <x:c r="F65" s="7" t="str">
+        <x:v>https://www.instagram.com/oxygenresidencecluj</x:v>
+      </x:c>
+      <x:c r="G65" s="7" t="str">
+        <x:v>https://www.facebook.com/oxygencluj</x:v>
+      </x:c>
+      <x:c r="H65" s="7"/>
+      <x:c r="I65" s="7" t="str">
+        <x:v>https://oxygencluj.ro/</x:v>
+      </x:c>
+      <x:c r="J65" s="13" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="K65" s="7" t="str">
+        <x:v>Dezvoltatori Cluj / Cluj-Napoca</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="66" ht="31.5" customHeight="1">
+      <x:c r="A66" s="7" t="str">
+        <x:v>Studium Green</x:v>
+      </x:c>
+      <x:c r="B66" s="7" t="str">
+        <x:v>Cluj</x:v>
+      </x:c>
+      <x:c r="C66" s="7" t="str">
+        <x:v>Str. Teodor Mihali, nr. 39-43, Cluj-Napoca</x:v>
+      </x:c>
+      <x:c r="D66" s="7" t="str">
+        <x:v>+40 788 421 669</x:v>
+      </x:c>
+      <x:c r="E66" s="7" t="str">
+        <x:v>https://www.studiumgreen.ro/</x:v>
+      </x:c>
+      <x:c r="F66" s="7" t="str">
+        <x:v>https://www.instagram.com/studium_green/</x:v>
+      </x:c>
+      <x:c r="G66" s="7" t="str">
+        <x:v>https://www.facebook.com/studiumgreenimobiliare/</x:v>
+      </x:c>
+      <x:c r="H66" s="7"/>
+      <x:c r="I66" s="7" t="str">
+        <x:v>https://www.studiumgreen.ro/</x:v>
+      </x:c>
+      <x:c r="J66" s="13" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="K66" s="7" t="str">
+        <x:v>Dezvoltatori Cluj / Cluj-Napoca</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="67" ht="31.5" customHeight="1">
+      <x:c r="A67" s="7" t="str">
+        <x:v>SDC Properties</x:v>
+      </x:c>
+      <x:c r="B67" s="7" t="str">
+        <x:v>Cluj</x:v>
+      </x:c>
+      <x:c r="C67" s="7" t="str">
+        <x:v>Str. Gheorghe Marinescu 36-38, Cluj-Napoca</x:v>
+      </x:c>
+      <x:c r="D67" s="7" t="str">
+        <x:v>+40 791 330 000</x:v>
+      </x:c>
+      <x:c r="E67" s="7" t="str">
+        <x:v>https://www.sdcproperties.ro/</x:v>
+      </x:c>
+      <x:c r="F67" s="7" t="str">
+        <x:v>https://www.instagram.com/sdc_properties</x:v>
+      </x:c>
+      <x:c r="G67" s="7" t="str">
+        <x:v>https://www.facebook.com/sdcproperty</x:v>
+      </x:c>
+      <x:c r="H67" s="7"/>
+      <x:c r="I67" s="7" t="str">
+        <x:v>https://www.sdcproperties.ro/</x:v>
+      </x:c>
+      <x:c r="J67" s="13" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="K67" s="7" t="str">
+        <x:v>Dezvoltatori Cluj / Cluj-Napoca</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="68" ht="31.5" customHeight="1">
+      <x:c r="A68" s="7" t="str">
+        <x:v>Transilvania Smart City</x:v>
+      </x:c>
+      <x:c r="B68" s="7" t="str">
+        <x:v>Cluj</x:v>
+      </x:c>
+      <x:c r="C68" s="7" t="str">
+        <x:v>Strada Moș Ion Roată 29, Cluj-Napoca</x:v>
+      </x:c>
+      <x:c r="D68" s="7" t="str">
+        <x:v>+40 790 330 000</x:v>
+      </x:c>
+      <x:c r="E68" s="7" t="str">
+        <x:v>https://www.transilvaniasmartcity.ro/</x:v>
+      </x:c>
+      <x:c r="F68" s="7" t="str">
+        <x:v>https://www.instagram.com/transilvaniasmartcity/</x:v>
+      </x:c>
+      <x:c r="G68" s="7" t="str">
+        <x:v>https://www.facebook.com/transilvania.smart.city</x:v>
+      </x:c>
+      <x:c r="H68" s="7"/>
+      <x:c r="I68" s="7" t="str">
+        <x:v>https://www.transilvaniasmartcity.ro/</x:v>
+      </x:c>
+      <x:c r="J68" s="13" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="K68" s="7" t="str">
+        <x:v>Dezvoltatori Cluj / Cluj-Napoca</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="69" ht="31.5" customHeight="1">
+      <x:c r="A69" s="7" t="str">
+        <x:v>Grand Park Sud Residence</x:v>
+      </x:c>
+      <x:c r="B69" s="7" t="str">
+        <x:v>Cluj</x:v>
+      </x:c>
+      <x:c r="C69" s="7" t="str">
+        <x:v>Strada Bună Ziua nr. 37, Cluj-Napoca</x:v>
+      </x:c>
+      <x:c r="D69" s="7" t="str">
+        <x:v>+40 753 053 203</x:v>
+      </x:c>
+      <x:c r="E69" s="7" t="str">
+        <x:v>https://www.grandparksudresidence.ro/</x:v>
+      </x:c>
+      <x:c r="F69" s="7"/>
+      <x:c r="G69" s="7" t="str">
+        <x:v>https://www.facebook.com/grandparksud</x:v>
+      </x:c>
+      <x:c r="H69" s="7"/>
+      <x:c r="I69" s="7" t="str">
+        <x:v>https://www.grandparksudresidence.ro/</x:v>
+      </x:c>
+      <x:c r="J69" s="13" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="K69" s="7" t="str">
+        <x:v>Dezvoltatori Cluj / Cluj-Napoca</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="70" ht="31.5" customHeight="1">
+      <x:c r="A70" s="7" t="str">
+        <x:v>CITIUS</x:v>
+      </x:c>
+      <x:c r="B70" s="7" t="str">
+        <x:v>Cluj</x:v>
+      </x:c>
+      <x:c r="C70" s="7" t="str">
+        <x:v>Strada Corneliu Coposu, nr. 167, Cluj-Napoca</x:v>
+      </x:c>
+      <x:c r="D70" s="7" t="str">
+        <x:v>+40 371 780 065</x:v>
+      </x:c>
+      <x:c r="E70" s="7" t="str">
+        <x:v>https://www.citius.ro/</x:v>
+      </x:c>
+      <x:c r="F70" s="7" t="str">
+        <x:v>https://www.instagram.com/citius_cluj/</x:v>
+      </x:c>
+      <x:c r="G70" s="7" t="str">
+        <x:v>https://www.facebook.com/profile.php?id=61557456396360</x:v>
+      </x:c>
+      <x:c r="H70" s="7"/>
+      <x:c r="I70" s="7" t="str">
+        <x:v>https://www.citius.ro/</x:v>
+      </x:c>
+      <x:c r="J70" s="13" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="K70" s="7" t="str">
+        <x:v>Dezvoltatori Cluj / Cluj-Napoca</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="71" ht="31.5" customHeight="1">
+      <x:c r="A71" s="7" t="str">
+        <x:v>Solaris Development</x:v>
+      </x:c>
+      <x:c r="B71" s="7" t="str">
+        <x:v>Cluj</x:v>
+      </x:c>
+      <x:c r="C71" s="7" t="str">
+        <x:v>Strada Burebista nr. 9, parter, Cluj-Napoca</x:v>
+      </x:c>
+      <x:c r="D71" s="7" t="str">
+        <x:v>+40 749 126 643</x:v>
+      </x:c>
+      <x:c r="E71" s="7" t="str">
+        <x:v>https://solarisdevelopment.ro/</x:v>
+      </x:c>
+      <x:c r="F71" s="7"/>
+      <x:c r="G71" s="7" t="str">
+        <x:v>https://www.facebook.com/SolarisRealEstateInvestments/</x:v>
+      </x:c>
+      <x:c r="H71" s="7"/>
+      <x:c r="I71" s="7" t="str">
+        <x:v>https://solarisdevelopment.ro/</x:v>
+      </x:c>
+      <x:c r="J71" s="13" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="K71" s="7" t="str">
+        <x:v>Dezvoltatori Cluj / Cluj-Napoca</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="72" ht="31.5" customHeight="1">
+      <x:c r="A72" s="7" t="str">
+        <x:v>SCALA Sopor</x:v>
+      </x:c>
+      <x:c r="B72" s="7" t="str">
+        <x:v>Cluj</x:v>
+      </x:c>
+      <x:c r="C72" s="7" t="str">
+        <x:v>Strada Soporului nr. 21, Cluj-Napoca</x:v>
+      </x:c>
+      <x:c r="D72" s="7" t="str">
+        <x:v>+40 371 781 764</x:v>
+      </x:c>
+      <x:c r="E72" s="7" t="str">
+        <x:v>https://www.scalasopor.ro/</x:v>
+      </x:c>
+      <x:c r="F72" s="7" t="str">
+        <x:v>https://www.instagram.com/scalasopor/</x:v>
+      </x:c>
+      <x:c r="G72" s="7" t="str">
+        <x:v>https://www.facebook.com/profile.php?id=61565507230976</x:v>
+      </x:c>
+      <x:c r="H72" s="7"/>
+      <x:c r="I72" s="7" t="str">
+        <x:v>https://www.scalasopor.ro/contact</x:v>
+      </x:c>
+      <x:c r="J72" s="13" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="K72" s="7" t="str">
+        <x:v>Dezvoltatori Cluj / Cluj-Napoca</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="73" ht="31.5" customHeight="1">
+      <x:c r="A73" s="7" t="str">
+        <x:v>Casa Dinainte</x:v>
+      </x:c>
+      <x:c r="B73" s="7" t="str">
+        <x:v>Cluj</x:v>
+      </x:c>
+      <x:c r="C73" s="7" t="str">
+        <x:v>Sălicea 102i, 407236 Sălicea</x:v>
+      </x:c>
+      <x:c r="D73" s="7" t="str">
+        <x:v>+40 725 595 937</x:v>
+      </x:c>
+      <x:c r="E73" s="7" t="str">
+        <x:v>https://www.casadinainte.ro/</x:v>
+      </x:c>
+      <x:c r="F73" s="7"/>
+      <x:c r="G73" s="7"/>
+      <x:c r="H73" s="7"/>
+      <x:c r="I73" s="7" t="str">
+        <x:v>https://www.casadinainte.ro/locatie</x:v>
+      </x:c>
+      <x:c r="J73" s="13" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="K73" s="7" t="str">
+        <x:v>Cluj / Sălicea-Ciurila</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="74" ht="31.5" customHeight="1">
+      <x:c r="A74" s="7" t="str">
+        <x:v>Casele cu Stuf</x:v>
+      </x:c>
+      <x:c r="B74" s="7" t="str">
+        <x:v>Cluj</x:v>
+      </x:c>
+      <x:c r="C74" s="7" t="str">
+        <x:v>Sălicea, Str. Principală nr. 88A, com. Ciurila</x:v>
+      </x:c>
+      <x:c r="D74" s="7" t="str">
+        <x:v>+40 770 523 997</x:v>
+      </x:c>
+      <x:c r="E74" s="7" t="str">
+        <x:v>https://www.caselecustuf.ro/</x:v>
+      </x:c>
+      <x:c r="F74" s="7"/>
+      <x:c r="G74" s="7"/>
+      <x:c r="H74" s="7"/>
+      <x:c r="I74" s="7" t="str">
+        <x:v>https://www.caselecustuf.ro/</x:v>
+      </x:c>
+      <x:c r="J74" s="13" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="K74" s="7" t="str">
+        <x:v>Cluj / Sălicea-Ciurila</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="75" ht="31.5" customHeight="1">
+      <x:c r="A75" s="7" t="str">
+        <x:v>Claudia Elkan / Pensiunea Amurg</x:v>
+      </x:c>
+      <x:c r="B75" s="7" t="str">
+        <x:v>Cluj</x:v>
+      </x:c>
+      <x:c r="C75" s="7" t="str">
+        <x:v>SAT SĂLICEA 136F, Sălicea</x:v>
+      </x:c>
+      <x:c r="D75" s="7" t="str">
+        <x:v>+40 723 577 670</x:v>
+      </x:c>
+      <x:c r="E75" s="7"/>
+      <x:c r="F75" s="7"/>
+      <x:c r="G75" s="7"/>
+      <x:c r="H75" s="7"/>
+      <x:c r="I75" s="7" t="str">
+        <x:v>https://www.booking.com/hotel/ro/pensiunea-amurg.ro.html</x:v>
+      </x:c>
+      <x:c r="J75" s="13" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="K75" s="7" t="str">
+        <x:v>Cluj / Sălicea-Ciurila</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="76" ht="31.5" customHeight="1">
+      <x:c r="A76" s="7" t="str">
+        <x:v>Camping Moara de Vânt / DND Travel</x:v>
+      </x:c>
+      <x:c r="B76" s="7" t="str">
+        <x:v>Cluj</x:v>
+      </x:c>
+      <x:c r="C76" s="7" t="str">
+        <x:v>Drum DC 91, Sălicea, 407236</x:v>
+      </x:c>
+      <x:c r="D76" s="7" t="str">
+        <x:v>+40 744 930 434</x:v>
+      </x:c>
+      <x:c r="E76" s="7" t="str">
+        <x:v>https://www.dndtravel.ro/moara-de-vant/</x:v>
+      </x:c>
+      <x:c r="F76" s="7"/>
+      <x:c r="G76" s="7"/>
+      <x:c r="H76" s="7"/>
+      <x:c r="I76" s="7" t="str">
+        <x:v>https://www.dndtravel.ro/moara-de-vant/</x:v>
+      </x:c>
+      <x:c r="J76" s="13" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="K76" s="7" t="str">
+        <x:v>Cluj / Sălicea-Ciurila</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="77" ht="31.5" customHeight="1">
+      <x:c r="A77" s="7" t="str">
+        <x:v>Domeniul Regilor / TIPOAVIAS SRL</x:v>
+      </x:c>
+      <x:c r="B77" s="7" t="str">
+        <x:v>Cluj</x:v>
+      </x:c>
+      <x:c r="C77" s="7" t="str">
+        <x:v>Ciurila nr. 147A, 407230 Ciurila</x:v>
+      </x:c>
+      <x:c r="D77" s="7" t="str">
+        <x:v>+40 732 124 247</x:v>
+      </x:c>
+      <x:c r="E77" s="7" t="str">
+        <x:v>https://domeniulregilor.ro/</x:v>
+      </x:c>
+      <x:c r="F77" s="7"/>
+      <x:c r="G77" s="7"/>
+      <x:c r="H77" s="7"/>
+      <x:c r="I77" s="7" t="str">
+        <x:v>https://beta.domeniulregilor.ro/rezervari/</x:v>
+      </x:c>
+      <x:c r="J77" s="13" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="K77" s="7" t="str">
+        <x:v>Cluj / Ciurila</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="78" ht="31.5" customHeight="1">
+      <x:c r="A78" s="7" t="str">
+        <x:v>Casa Barolo</x:v>
+      </x:c>
+      <x:c r="B78" s="7" t="str">
+        <x:v>Cluj</x:v>
+      </x:c>
+      <x:c r="C78" s="7" t="str">
+        <x:v>Str. Principală nr. 358, Vlaha, Com. Săvădisla</x:v>
+      </x:c>
+      <x:c r="D78" s="7" t="str">
+        <x:v>+40 734 771 140</x:v>
+      </x:c>
+      <x:c r="E78" s="7" t="str">
+        <x:v>https://casabarolo.ro/</x:v>
+      </x:c>
+      <x:c r="F78" s="7"/>
+      <x:c r="G78" s="7" t="str">
+        <x:v>https://www.facebook.com/CasaBaroloVlaha</x:v>
+      </x:c>
+      <x:c r="H78" s="7"/>
+      <x:c r="I78" s="7" t="str">
+        <x:v>https://casabarolo.ro/contact/</x:v>
+      </x:c>
+      <x:c r="J78" s="13" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="K78" s="7" t="str">
+        <x:v>Cluj / Săvădisla-Vlaha</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="79" ht="31.5" customHeight="1">
+      <x:c r="A79" s="7" t="str">
+        <x:v>Copfos csárda</x:v>
+      </x:c>
+      <x:c r="B79" s="7" t="str">
+        <x:v>Cluj</x:v>
+      </x:c>
+      <x:c r="C79" s="7" t="str">
+        <x:v>Săvădisla nr. 151</x:v>
+      </x:c>
+      <x:c r="D79" s="7" t="str">
+        <x:v>+40 742 053 700</x:v>
+      </x:c>
+      <x:c r="E79" s="7"/>
+      <x:c r="F79" s="7"/>
+      <x:c r="G79" s="7" t="str">
+        <x:v>https://www.facebook.com/copfoscsarda</x:v>
+      </x:c>
+      <x:c r="H79" s="7"/>
+      <x:c r="I79" s="7" t="str">
+        <x:v>https://www.welcometoromania.ro/E60_Oradea_Cluj/E60_Oradea_Cluj_Savadisla_Copfos_Csarda_r.htm</x:v>
+      </x:c>
+      <x:c r="J79" s="13" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="K79" s="7" t="str">
+        <x:v>Cluj / Săvădisla</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="80" ht="31.5" customHeight="1">
+      <x:c r="A80" s="7" t="str">
+        <x:v>Pensiunea La Conac</x:v>
+      </x:c>
+      <x:c r="B80" s="7" t="str">
+        <x:v>Cluj</x:v>
+      </x:c>
+      <x:c r="C80" s="7" t="str">
+        <x:v>Săliștea Veche nr. 3, 407212 Săliștea Veche</x:v>
+      </x:c>
+      <x:c r="D80" s="7" t="str">
+        <x:v>+40 728 010 757</x:v>
+      </x:c>
+      <x:c r="E80" s="7"/>
+      <x:c r="F80" s="7"/>
+      <x:c r="G80" s="7"/>
+      <x:c r="H80" s="7"/>
+      <x:c r="I80" s="7" t="str">
+        <x:v>https://www.booking.com/hotel/ro/pensiunea-la-conac.ro.html</x:v>
+      </x:c>
+      <x:c r="J80" s="13" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="K80" s="7" t="str">
+        <x:v>Cluj / Chinteni-Săliștea Veche</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="81" ht="31.5" customHeight="1">
+      <x:c r="A81" s="7" t="str">
+        <x:v>Casa Thor</x:v>
+      </x:c>
+      <x:c r="B81" s="7" t="str">
+        <x:v>Cluj</x:v>
+      </x:c>
+      <x:c r="C81" s="7" t="str">
+        <x:v>Localitatea Dângău Mic, 407151</x:v>
+      </x:c>
+      <x:c r="D81" s="7" t="str">
+        <x:v>+40 770 441 378</x:v>
+      </x:c>
+      <x:c r="E81" s="7" t="str">
+        <x:v>https://casathor.ro/</x:v>
+      </x:c>
+      <x:c r="F81" s="7"/>
+      <x:c r="G81" s="7"/>
+      <x:c r="H81" s="7"/>
+      <x:c r="I81" s="7" t="str">
+        <x:v>https://casathor.ro/servicii-cabana-mare/</x:v>
+      </x:c>
+      <x:c r="J81" s="13" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="K81" s="7" t="str">
+        <x:v>Cluj / Dângău-Căpușu Mare</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="82" ht="31.5" customHeight="1">
+      <x:c r="A82" s="7" t="str">
+        <x:v>Pensiunea Casa Stan</x:v>
+      </x:c>
+      <x:c r="B82" s="7" t="str">
+        <x:v>Cluj</x:v>
+      </x:c>
+      <x:c r="C82" s="7" t="str">
+        <x:v>Str. Principală nr. 87B, Dângău Mare</x:v>
+      </x:c>
+      <x:c r="D82" s="7" t="str">
+        <x:v>+40 743 571 461</x:v>
+      </x:c>
+      <x:c r="E82" s="7" t="str">
+        <x:v>https://pensiuneacasastancluj.ro/</x:v>
+      </x:c>
+      <x:c r="F82" s="7"/>
+      <x:c r="G82" s="7"/>
+      <x:c r="H82" s="7"/>
+      <x:c r="I82" s="7" t="str">
+        <x:v>https://pensiuneacasastancluj.ro/</x:v>
+      </x:c>
+      <x:c r="J82" s="13" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="K82" s="7" t="str">
+        <x:v>Cluj / Dângău-Căpușu Mare</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="83" ht="31.5" customHeight="1">
+      <x:c r="A83" s="7" t="str">
+        <x:v>Cuib 176</x:v>
+      </x:c>
+      <x:c r="B83" s="7" t="str">
+        <x:v>Cluj</x:v>
+      </x:c>
+      <x:c r="C83" s="7" t="str">
+        <x:v>Căpușu Mic, Str. Principală nr. 176A</x:v>
+      </x:c>
+      <x:c r="D83" s="7" t="str">
+        <x:v>+40 724 143 849</x:v>
+      </x:c>
+      <x:c r="E83" s="7" t="str">
+        <x:v>https://www.cuib176.ro/</x:v>
+      </x:c>
+      <x:c r="F83" s="7"/>
+      <x:c r="G83" s="7"/>
+      <x:c r="H83" s="7"/>
+      <x:c r="I83" s="7" t="str">
+        <x:v>https://clujtourism.ro/pensiuni-agroturistice-cluj/</x:v>
+      </x:c>
+      <x:c r="J83" s="13" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="K83" s="7" t="str">
+        <x:v>Cluj / Căpușu Mic</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="84" ht="31.5" customHeight="1">
+      <x:c r="A84" s="7" t="str">
+        <x:v>Pensiunea Energy</x:v>
+      </x:c>
+      <x:c r="B84" s="7" t="str">
+        <x:v>Cluj</x:v>
+      </x:c>
+      <x:c r="C84" s="7" t="str">
+        <x:v>Strada Principală 260, 407148 Căpușu Mic</x:v>
+      </x:c>
+      <x:c r="D84" s="7" t="str">
+        <x:v>+40 752 152 570</x:v>
+      </x:c>
+      <x:c r="E84" s="7" t="str">
+        <x:v>https://www.pensiuneaenergy.ro/</x:v>
+      </x:c>
+      <x:c r="F84" s="7"/>
+      <x:c r="G84" s="7"/>
+      <x:c r="H84" s="7"/>
+      <x:c r="I84" s="7" t="str">
+        <x:v>https://www.booking.com/hotel/ro/pensiunea-energy.ro.html</x:v>
+      </x:c>
+      <x:c r="J84" s="13" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="K84" s="7" t="str">
+        <x:v>Cluj / Căpușu Mic</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="85" ht="31.5" customHeight="1">
+      <x:c r="A85" s="7" t="str">
+        <x:v>Pensiunea Frații Iancu</x:v>
+      </x:c>
+      <x:c r="B85" s="7" t="str">
+        <x:v>Cluj</x:v>
+      </x:c>
+      <x:c r="C85" s="7" t="str">
+        <x:v>Dumbrava nr. 260, Căpușu Mare</x:v>
+      </x:c>
+      <x:c r="D85" s="7" t="str">
+        <x:v>+40 740 914 176</x:v>
+      </x:c>
+      <x:c r="E85" s="7" t="str">
+        <x:v>https://www.pensiuneafratiiiancu.ro/</x:v>
+      </x:c>
+      <x:c r="F85" s="7"/>
+      <x:c r="G85" s="7"/>
+      <x:c r="H85" s="7"/>
+      <x:c r="I85" s="7" t="str">
+        <x:v>https://www.airbnb.it/rooms/817797212040092657</x:v>
+      </x:c>
+      <x:c r="J85" s="13" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="K85" s="7" t="str">
+        <x:v>Cluj / Căpușu Mare-Dumbrava</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="86" ht="31.5" customHeight="1">
+      <x:c r="A86" s="7" t="str">
+        <x:v>Complex Turistic Căpuș</x:v>
+      </x:c>
+      <x:c r="B86" s="7" t="str">
+        <x:v>Cluj</x:v>
+      </x:c>
+      <x:c r="C86" s="7" t="str">
+        <x:v>DN1, 407145 Căpușu Mare</x:v>
+      </x:c>
+      <x:c r="D86" s="7" t="str">
+        <x:v>+40 741 264 330</x:v>
+      </x:c>
+      <x:c r="E86" s="7" t="str">
+        <x:v>https://complexturisticcapus.eatbu.com/?lang=en</x:v>
+      </x:c>
+      <x:c r="F86" s="7"/>
+      <x:c r="G86" s="7"/>
+      <x:c r="H86" s="7"/>
+      <x:c r="I86" s="7" t="str">
+        <x:v>https://complexturisticcapus.eatbu.com/?lang=en</x:v>
+      </x:c>
+      <x:c r="J86" s="13" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="K86" s="7" t="str">
+        <x:v>Cluj / Căpușu Mare</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="87" ht="31.5" customHeight="1">
+      <x:c r="A87" s="7" t="str">
+        <x:v>Casa Maria - Valea Drăganului</x:v>
+      </x:c>
+      <x:c r="B87" s="7" t="str">
+        <x:v>Cluj</x:v>
+      </x:c>
+      <x:c r="C87" s="7" t="str">
+        <x:v>Lunca Vișagului 123A, 407474</x:v>
+      </x:c>
+      <x:c r="D87" s="7" t="str">
+        <x:v>+40 744 404 434</x:v>
+      </x:c>
+      <x:c r="E87" s="7" t="str">
+        <x:v>https://valea-draganului.ro/</x:v>
+      </x:c>
+      <x:c r="F87" s="7"/>
+      <x:c r="G87" s="7"/>
+      <x:c r="H87" s="7"/>
+      <x:c r="I87" s="7" t="str">
+        <x:v>https://valea-draganului.ro/</x:v>
+      </x:c>
+      <x:c r="J87" s="13" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="K87" s="7" t="str">
+        <x:v>Cluj / Valea Drăganului-Poieni</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="88" ht="31.5" customHeight="1">
+      <x:c r="A88" s="7" t="str">
+        <x:v>Casa Morar - Cabana 1</x:v>
+      </x:c>
+      <x:c r="B88" s="7" t="str">
+        <x:v>Cluj</x:v>
+      </x:c>
+      <x:c r="C88" s="7" t="str">
+        <x:v>Valea Drăganului nr. 226, com. Poieni</x:v>
+      </x:c>
+      <x:c r="D88" s="7" t="str">
+        <x:v>+40 727 791 271</x:v>
+      </x:c>
+      <x:c r="E88" s="7" t="str">
+        <x:v>https://casamorar.ro/</x:v>
+      </x:c>
+      <x:c r="F88" s="7"/>
+      <x:c r="G88" s="7" t="str">
+        <x:v>https://www.facebook.com/pages/Pensiunea-Casa-Morar-Valea-Draganului/174431915910804</x:v>
+      </x:c>
+      <x:c r="H88" s="7"/>
+      <x:c r="I88" s="7" t="str">
+        <x:v>https://casamorar.ro/cabana-1/</x:v>
+      </x:c>
+      <x:c r="J88" s="13" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="K88" s="7" t="str">
+        <x:v>Cluj / Valea Drăganului-Poieni</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="89" ht="31.5" customHeight="1">
+      <x:c r="A89" s="7" t="str">
+        <x:v>Cabana Drăgana</x:v>
+      </x:c>
+      <x:c r="B89" s="7" t="str">
+        <x:v>Cluj</x:v>
+      </x:c>
+      <x:c r="C89" s="7" t="str">
+        <x:v>Principala 29C, Lunca Vișagului, 407474</x:v>
+      </x:c>
+      <x:c r="D89" s="7" t="str">
+        <x:v>+40 740 901 604</x:v>
+      </x:c>
+      <x:c r="E89" s="7" t="str">
+        <x:v>https://dragana.ro/</x:v>
+      </x:c>
+      <x:c r="F89" s="7"/>
+      <x:c r="G89" s="7"/>
+      <x:c r="H89" s="7"/>
+      <x:c r="I89" s="7" t="str">
+        <x:v>https://dragana.ro/</x:v>
+      </x:c>
+      <x:c r="J89" s="13" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="K89" s="7" t="str">
+        <x:v>Cluj / Valea Drăganului-Poieni</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="90" ht="31.5" customHeight="1">
+      <x:c r="A90" s="7" t="str">
+        <x:v>Cabana Iubu</x:v>
+      </x:c>
+      <x:c r="B90" s="7" t="str">
+        <x:v>Cluj</x:v>
+      </x:c>
+      <x:c r="C90" s="7" t="str">
+        <x:v>Valea Drăganului</x:v>
+      </x:c>
+      <x:c r="D90" s="7" t="str">
+        <x:v>+40 724 336 966</x:v>
+      </x:c>
+      <x:c r="E90" s="7" t="str">
+        <x:v>https://cabanaiubu.ro/</x:v>
+      </x:c>
+      <x:c r="F90" s="7"/>
+      <x:c r="G90" s="7"/>
+      <x:c r="H90" s="7"/>
+      <x:c r="I90" s="7" t="str">
+        <x:v>https://cabanaiubu.ro/despre/</x:v>
+      </x:c>
+      <x:c r="J90" s="13" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="K90" s="7" t="str">
+        <x:v>Cluj / Valea Drăganului-Poieni</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="91" ht="31.5" customHeight="1">
+      <x:c r="A91" s="7" t="str">
+        <x:v>Cabana La Frăguțe</x:v>
+      </x:c>
+      <x:c r="B91" s="7" t="str">
+        <x:v>Cluj</x:v>
+      </x:c>
+      <x:c r="C91" s="7" t="str">
+        <x:v>Valea Drăganului</x:v>
+      </x:c>
+      <x:c r="D91" s="7" t="str">
+        <x:v>+40 745 231 035</x:v>
+      </x:c>
+      <x:c r="E91" s="7"/>
+      <x:c r="F91" s="7"/>
+      <x:c r="G91" s="7"/>
+      <x:c r="H91" s="7"/>
+      <x:c r="I91" s="7" t="str">
+        <x:v>https://www.lapensiuni.ro/cabane-transilvania/cluj/valea-draganului</x:v>
+      </x:c>
+      <x:c r="J91" s="13" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="K91" s="7" t="str">
+        <x:v>Cluj / Valea Drăganului-Poieni</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="92" ht="31.5" customHeight="1">
+      <x:c r="A92" s="7" t="str">
+        <x:v>Cabana Vlădeasa</x:v>
+      </x:c>
+      <x:c r="B92" s="7" t="str">
+        <x:v>Cluj</x:v>
+      </x:c>
+      <x:c r="C92" s="7" t="str">
+        <x:v>Rogojel 161A, 407496</x:v>
+      </x:c>
+      <x:c r="D92" s="7" t="str">
+        <x:v>+40 743 062 378</x:v>
+      </x:c>
+      <x:c r="E92" s="7"/>
+      <x:c r="F92" s="7"/>
+      <x:c r="G92" s="7"/>
+      <x:c r="H92" s="7"/>
+      <x:c r="I92" s="7" t="str">
+        <x:v>https://webcamromania.ro/webcam-munte/webcam-cabana-vladeasa/</x:v>
+      </x:c>
+      <x:c r="J92" s="13" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="K92" s="7" t="str">
+        <x:v>Cluj / Rogojel-Săcuieu</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="93" ht="31.5" customHeight="1">
+      <x:c r="A93" s="7" t="str">
+        <x:v>Cabana Ruth</x:v>
+      </x:c>
+      <x:c r="B93" s="7" t="str">
+        <x:v>Cluj</x:v>
+      </x:c>
+      <x:c r="C93" s="7" t="str">
+        <x:v>Valea Ierii nr. 275P</x:v>
+      </x:c>
+      <x:c r="D93" s="7" t="str">
+        <x:v>+40 742 965 252</x:v>
+      </x:c>
+      <x:c r="E93" s="7" t="str">
+        <x:v>https://www.cabanaruth.ro/</x:v>
+      </x:c>
+      <x:c r="F93" s="7"/>
+      <x:c r="G93" s="7"/>
+      <x:c r="H93" s="7"/>
+      <x:c r="I93" s="7" t="str">
+        <x:v>https://www.cabanaruth.ro/</x:v>
+      </x:c>
+      <x:c r="J93" s="13" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="K93" s="7" t="str">
+        <x:v>Cluj / Valea Ierii</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="94" ht="31.5" customHeight="1">
+      <x:c r="A94" s="7" t="str">
+        <x:v>Cabana Valea Ierii Home</x:v>
+      </x:c>
+      <x:c r="B94" s="7" t="str">
+        <x:v>Cluj</x:v>
+      </x:c>
+      <x:c r="C94" s="7" t="str">
+        <x:v>Str. Principală nr. 2F, Valea Ierii</x:v>
+      </x:c>
+      <x:c r="D94" s="7" t="str">
+        <x:v>+40 758 937 205</x:v>
+      </x:c>
+      <x:c r="E94" s="7"/>
+      <x:c r="F94" s="7"/>
+      <x:c r="G94" s="7"/>
+      <x:c r="H94" s="7"/>
+      <x:c r="I94" s="7" t="str">
+        <x:v>https://www.turistinfo.ro/valea_ierii/cazare-valea_ierii/cabana_valea_ierii_home-c118225.html</x:v>
+      </x:c>
+      <x:c r="J94" s="13" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="K94" s="7" t="str">
+        <x:v>Cluj / Valea Ierii</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="95" ht="31.5" customHeight="1">
+      <x:c r="A95" s="7" t="str">
+        <x:v>Pensiunea Lara&amp;Mara</x:v>
+      </x:c>
+      <x:c r="B95" s="7" t="str">
+        <x:v>Cluj</x:v>
+      </x:c>
+      <x:c r="C95" s="7" t="str">
+        <x:v>DJ107N, Valea Ierii</x:v>
+      </x:c>
+      <x:c r="D95" s="7" t="str">
+        <x:v>+40 756 394 933</x:v>
+      </x:c>
+      <x:c r="E95" s="7" t="str">
+        <x:v>https://www.pensiunealara.com/</x:v>
+      </x:c>
+      <x:c r="F95" s="7"/>
+      <x:c r="G95" s="7"/>
+      <x:c r="H95" s="7"/>
+      <x:c r="I95" s="7" t="str">
+        <x:v>https://www.turismvaleaierii.ro/en/cazari-si-servicii</x:v>
+      </x:c>
+      <x:c r="J95" s="13" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="K95" s="7" t="str">
+        <x:v>Cluj / Valea Ierii</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="96" ht="31.5" customHeight="1">
+      <x:c r="A96" s="7" t="str">
+        <x:v>Casa Călățele</x:v>
+      </x:c>
+      <x:c r="B96" s="7" t="str">
+        <x:v>Cluj</x:v>
+      </x:c>
+      <x:c r="C96" s="7" t="str">
+        <x:v>Călățele-Pădure nr. 534, comuna Călățele</x:v>
+      </x:c>
+      <x:c r="D96" s="7" t="str">
+        <x:v>+40 734 771 177</x:v>
+      </x:c>
+      <x:c r="E96" s="7" t="str">
+        <x:v>http://universt.ro/</x:v>
+      </x:c>
+      <x:c r="F96" s="7"/>
+      <x:c r="G96" s="7"/>
+      <x:c r="H96" s="7"/>
+      <x:c r="I96" s="7" t="str">
+        <x:v>https://cluj.com/cazare/casa-calatele-cazare-judetul-cluj/</x:v>
+      </x:c>
+      <x:c r="J96" s="13" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="K96" s="7" t="str">
+        <x:v>Cluj / Călățele</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="97" ht="31.5" customHeight="1">
+      <x:c r="A97" s="7" t="str">
+        <x:v>drag de apuseni</x:v>
+      </x:c>
+      <x:c r="B97" s="7" t="str">
+        <x:v>Cluj</x:v>
+      </x:c>
+      <x:c r="C97" s="7" t="str">
+        <x:v>Sat de Vacanță I nr. 143, Călățele</x:v>
+      </x:c>
+      <x:c r="D97" s="7" t="str">
+        <x:v>+40 745 254 118</x:v>
+      </x:c>
+      <x:c r="E97" s="7" t="str">
+        <x:v>https://www.dragdeapuseni.ro/</x:v>
+      </x:c>
+      <x:c r="F97" s="7"/>
+      <x:c r="G97" s="7"/>
+      <x:c r="H97" s="7"/>
+      <x:c r="I97" s="7" t="str">
+        <x:v>https://www.google.ro/travel/hotels/entity/ChkI973ehqWO54kTGg0vZy8xMWp0dF9iNTJuEAE</x:v>
+      </x:c>
+      <x:c r="J97" s="13" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="K97" s="7" t="str">
+        <x:v>Cluj / Călățele</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="98" ht="31.5" customHeight="1">
+      <x:c r="A98" s="7" t="str">
+        <x:v>Cazare Pensiune Sancraiu - Saroklak Póka Erzsébet</x:v>
+      </x:c>
+      <x:c r="B98" s="7" t="str">
+        <x:v>Cluj</x:v>
+      </x:c>
+      <x:c r="C98" s="7" t="str">
+        <x:v>Strada Principală 170, Sâncraiu, 407515</x:v>
+      </x:c>
+      <x:c r="D98" s="7" t="str">
+        <x:v>+40 742 050 702</x:v>
+      </x:c>
+      <x:c r="E98" s="7" t="str">
+        <x:v>http://saroklak.xtadia.com</x:v>
+      </x:c>
+      <x:c r="F98" s="7"/>
+      <x:c r="G98" s="7"/>
+      <x:c r="H98" s="7"/>
+      <x:c r="I98" s="7" t="str">
+        <x:v>https://sancraiu.cylex.ro/firma/cazare%2Bpensiune%2Bsancraiu%2B-%2Bsaroklak%2Bpoka%2Berzs%C3%A9bet-1322546.html</x:v>
+      </x:c>
+      <x:c r="J98" s="13" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="K98" s="7" t="str">
+        <x:v>Cluj / Sâncraiu</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="99" ht="31.5" customHeight="1">
+      <x:c r="A99" s="7" t="str">
+        <x:v>Pensiunea Tip-Top</x:v>
+      </x:c>
+      <x:c r="B99" s="7" t="str">
+        <x:v>Cluj</x:v>
+      </x:c>
+      <x:c r="C99" s="7" t="str">
+        <x:v>Str. Principală nr. 304, Sâncraiu, 407515</x:v>
+      </x:c>
+      <x:c r="D99" s="7" t="str">
+        <x:v>+40 741 103 653</x:v>
+      </x:c>
+      <x:c r="E99" s="7" t="str">
+        <x:v>https://pensiuneatiptop.cazare7.ro/contact</x:v>
+      </x:c>
+      <x:c r="F99" s="7"/>
+      <x:c r="G99" s="7"/>
+      <x:c r="H99" s="7"/>
+      <x:c r="I99" s="7" t="str">
+        <x:v>https://pensiuneatiptop.cazare7.ro/contact</x:v>
+      </x:c>
+      <x:c r="J99" s="13" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="K99" s="7" t="str">
+        <x:v>Cluj / Sâncraiu</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="100" ht="31.5" customHeight="1">
+      <x:c r="A100" s="7" t="str">
+        <x:v>hanul de vis</x:v>
+      </x:c>
+      <x:c r="B100" s="7" t="str">
+        <x:v>Cluj</x:v>
+      </x:c>
+      <x:c r="C100" s="7" t="str">
+        <x:v>Călățele-Pădure nr. 589</x:v>
+      </x:c>
+      <x:c r="D100" s="7" t="str">
+        <x:v>+40 747 082 653</x:v>
+      </x:c>
+      <x:c r="E100" s="7" t="str">
+        <x:v>https://www.hanuldevis.ro/</x:v>
+      </x:c>
+      <x:c r="F100" s="7"/>
+      <x:c r="G100" s="7"/>
+      <x:c r="H100" s="7"/>
+      <x:c r="I100" s="7" t="str">
+        <x:v>https://clujtourism.ro/pensiuni-agroturistice-cluj/</x:v>
+      </x:c>
+      <x:c r="J100" s="13" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="K100" s="7" t="str">
+        <x:v>Cluj / Călățele</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="101" ht="31.5" customHeight="1">
+      <x:c r="A101" s="7" t="str">
+        <x:v>Steaua Apusenilor</x:v>
+      </x:c>
+      <x:c r="B101" s="7" t="str">
+        <x:v>Cluj</x:v>
+      </x:c>
+      <x:c r="C101" s="7" t="str">
+        <x:v>Călățele-Pădure nr. 586A</x:v>
+      </x:c>
+      <x:c r="D101" s="7" t="str">
+        <x:v>+40 757 405 523</x:v>
+      </x:c>
+      <x:c r="E101" s="7"/>
+      <x:c r="F101" s="7"/>
+      <x:c r="G101" s="7"/>
+      <x:c r="H101" s="7"/>
+      <x:c r="I101" s="7" t="str">
+        <x:v>https://clujtourism.ro/pensiuni-agroturistice-cluj/</x:v>
+      </x:c>
+      <x:c r="J101" s="13" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="K101" s="7" t="str">
+        <x:v>Cluj / Călățele</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="102" ht="31.5" customHeight="1">
+      <x:c r="A102" s="7" t="str">
+        <x:v>casa olivia</x:v>
+      </x:c>
+      <x:c r="B102" s="7" t="str">
+        <x:v>Cluj</x:v>
+      </x:c>
+      <x:c r="C102" s="7" t="str">
+        <x:v>Călățele nr. 517</x:v>
+      </x:c>
+      <x:c r="D102" s="7" t="str">
+        <x:v>+40 764 399 609</x:v>
+      </x:c>
+      <x:c r="E102" s="7"/>
+      <x:c r="F102" s="7"/>
+      <x:c r="G102" s="7"/>
+      <x:c r="H102" s="7"/>
+      <x:c r="I102" s="7" t="str">
+        <x:v>https://clujtourism.ro/pensiuni-agroturistice-cluj/</x:v>
+      </x:c>
+      <x:c r="J102" s="13" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="K102" s="7" t="str">
+        <x:v>Cluj / Călățele</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="103" ht="31.5" customHeight="1">
+      <x:c r="A103" s="7" t="str">
+        <x:v>carmina</x:v>
+      </x:c>
+      <x:c r="B103" s="7" t="str">
+        <x:v>Cluj</x:v>
+      </x:c>
+      <x:c r="C103" s="7" t="str">
+        <x:v>Călățele / Dealul Negru nr. 75</x:v>
+      </x:c>
+      <x:c r="D103" s="7" t="str">
+        <x:v>+40 755 247 756</x:v>
+      </x:c>
+      <x:c r="E103" s="7"/>
+      <x:c r="F103" s="7"/>
+      <x:c r="G103" s="7"/>
+      <x:c r="H103" s="7"/>
+      <x:c r="I103" s="7" t="str">
+        <x:v>https://clujtourism.ro/pensiuni-agroturistice-cluj/</x:v>
+      </x:c>
+      <x:c r="J103" s="13" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="K103" s="7" t="str">
+        <x:v>Cluj / Călățele-Dealul Negru</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="104" ht="31.5" customHeight="1">
+      <x:c r="A104" s="7" t="str">
+        <x:v>La Stan</x:v>
+      </x:c>
+      <x:c r="B104" s="7" t="str">
+        <x:v>Cluj</x:v>
+      </x:c>
+      <x:c r="C104" s="7" t="str">
+        <x:v>Călățele nr. 86</x:v>
+      </x:c>
+      <x:c r="D104" s="7" t="str">
+        <x:v>+40 749 189 141</x:v>
+      </x:c>
+      <x:c r="E104" s="7"/>
+      <x:c r="F104" s="7"/>
+      <x:c r="G104" s="7"/>
+      <x:c r="H104" s="7"/>
+      <x:c r="I104" s="7" t="str">
+        <x:v>https://clujtourism.ro/pensiuni-agroturistice-cluj/</x:v>
+      </x:c>
+      <x:c r="J104" s="13" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="K104" s="7" t="str">
+        <x:v>Cluj / Călățele</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="105" ht="31.5" customHeight="1">
+      <x:c r="A105" s="7" t="str">
+        <x:v>Casa Bica</x:v>
+      </x:c>
+      <x:c r="B105" s="7" t="str">
+        <x:v>Cluj</x:v>
+      </x:c>
+      <x:c r="C105" s="7" t="str">
+        <x:v>Cacova Ierii nr. 126, Iara</x:v>
+      </x:c>
+      <x:c r="D105" s="7" t="str">
+        <x:v>+40 745 960 731</x:v>
+      </x:c>
+      <x:c r="E105" s="7"/>
+      <x:c r="F105" s="7"/>
+      <x:c r="G105" s="7"/>
+      <x:c r="H105" s="7"/>
+      <x:c r="I105" s="7" t="str">
+        <x:v>https://clujtourism.ro/pensiuni-agroturistice-cluj/</x:v>
+      </x:c>
+      <x:c r="J105" s="13" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="K105" s="7" t="str">
+        <x:v>Cluj / Iara-Cacova Ierii</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="106" ht="31.5" customHeight="1">
+      <x:c r="A106" s="7" t="str">
+        <x:v>Cheile Apusenilor</x:v>
+      </x:c>
+      <x:c r="B106" s="7" t="str">
+        <x:v>Cluj</x:v>
+      </x:c>
+      <x:c r="C106" s="7" t="str">
+        <x:v>Săndulești nr. 382</x:v>
+      </x:c>
+      <x:c r="D106" s="7" t="str">
+        <x:v>+40 742 104 813</x:v>
+      </x:c>
+      <x:c r="E106" s="7" t="str">
+        <x:v>https://www.pensiuneacheileapusenilor.ro/</x:v>
+      </x:c>
+      <x:c r="F106" s="7"/>
+      <x:c r="G106" s="7"/>
+      <x:c r="H106" s="7"/>
+      <x:c r="I106" s="7" t="str">
+        <x:v>https://clujtourism.ro/pensiuni-agroturistice-cluj/</x:v>
+      </x:c>
+      <x:c r="J106" s="13" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="K106" s="7" t="str">
+        <x:v>Cluj / Săndulești</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="107" ht="31.5" customHeight="1">
+      <x:c r="A107" s="7" t="str">
+        <x:v>Eden</x:v>
+      </x:c>
+      <x:c r="B107" s="7" t="str">
+        <x:v>Cluj</x:v>
+      </x:c>
+      <x:c r="C107" s="7" t="str">
+        <x:v>Săndulești / Copăceni nr. 327</x:v>
+      </x:c>
+      <x:c r="D107" s="7" t="str">
+        <x:v>+40 785 204 233</x:v>
+      </x:c>
+      <x:c r="E107" s="7" t="str">
+        <x:v>https://www.pensiuneaeden.ro/</x:v>
+      </x:c>
+      <x:c r="F107" s="7"/>
+      <x:c r="G107" s="7"/>
+      <x:c r="H107" s="7"/>
+      <x:c r="I107" s="7" t="str">
+        <x:v>https://clujtourism.ro/pensiuni-agroturistice-cluj/</x:v>
+      </x:c>
+      <x:c r="J107" s="13" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="K107" s="7" t="str">
+        <x:v>Cluj / Săndulești-Copăceni</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="108" ht="31.5" customHeight="1">
+      <x:c r="A108" s="7" t="str">
+        <x:v>Roa</x:v>
+      </x:c>
+      <x:c r="B108" s="7" t="str">
+        <x:v>Cluj</x:v>
+      </x:c>
+      <x:c r="C108" s="7" t="str">
+        <x:v>Săndulești nr. 1B</x:v>
+      </x:c>
+      <x:c r="D108" s="7" t="str">
+        <x:v>+40 770 467 544</x:v>
+      </x:c>
+      <x:c r="E108" s="7" t="str">
+        <x:v>https://www.laroa.ro/</x:v>
+      </x:c>
+      <x:c r="F108" s="7"/>
+      <x:c r="G108" s="7"/>
+      <x:c r="H108" s="7"/>
+      <x:c r="I108" s="7" t="str">
+        <x:v>https://clujtourism.ro/pensiuni-agroturistice-cluj/</x:v>
+      </x:c>
+      <x:c r="J108" s="13" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="K108" s="7" t="str">
+        <x:v>Cluj / Săndulești</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="109" ht="31.5" customHeight="1">
+      <x:c r="A109" s="7" t="str">
+        <x:v>Casa din Vale</x:v>
+      </x:c>
+      <x:c r="B109" s="7" t="str">
+        <x:v>Cluj</x:v>
+      </x:c>
+      <x:c r="C109" s="7" t="str">
+        <x:v>Săcuieu nr. 7</x:v>
+      </x:c>
+      <x:c r="D109" s="7" t="str">
+        <x:v>+40 742 782 376</x:v>
+      </x:c>
+      <x:c r="E109" s="7" t="str">
+        <x:v>https://www.casa-din-vale.ro/</x:v>
+      </x:c>
+      <x:c r="F109" s="7"/>
+      <x:c r="G109" s="7"/>
+      <x:c r="H109" s="7"/>
+      <x:c r="I109" s="7" t="str">
+        <x:v>https://clujtourism.ro/pensiuni-agroturistice-cluj/</x:v>
+      </x:c>
+      <x:c r="J109" s="13" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="K109" s="7" t="str">
+        <x:v>Cluj / Săcuieu</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="110" ht="31.5" customHeight="1">
+      <x:c r="A110" s="7" t="str">
+        <x:v>MORĂRIȚA</x:v>
+      </x:c>
+      <x:c r="B110" s="7" t="str">
+        <x:v>Cluj</x:v>
+      </x:c>
+      <x:c r="C110" s="7" t="str">
+        <x:v>Bonțida, str. Cotuțiului nr. 841</x:v>
+      </x:c>
+      <x:c r="D110" s="7" t="str">
+        <x:v>+40 757 038 886</x:v>
+      </x:c>
+      <x:c r="E110" s="7" t="str">
+        <x:v>https://www.pensiuneamorarita.ro/</x:v>
+      </x:c>
+      <x:c r="F110" s="7"/>
+      <x:c r="G110" s="7"/>
+      <x:c r="H110" s="7"/>
+      <x:c r="I110" s="7" t="str">
+        <x:v>https://clujtourism.ro/pensiuni-agroturistice-cluj/</x:v>
+      </x:c>
+      <x:c r="J110" s="13" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="K110" s="7" t="str">
+        <x:v>Cluj / Bonțida</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="111" ht="31.5" customHeight="1">
+      <x:c r="A111" s="7" t="str">
+        <x:v>Pensiunea Sipos Lidia</x:v>
+      </x:c>
+      <x:c r="B111" s="7" t="str">
+        <x:v>Cluj</x:v>
+      </x:c>
+      <x:c r="C111" s="7" t="str">
+        <x:v>Valea Ierii nr. 56</x:v>
+      </x:c>
+      <x:c r="D111" s="7" t="str">
+        <x:v>+40 747 409 381</x:v>
+      </x:c>
+      <x:c r="E111" s="7" t="str">
+        <x:v>https://cazare-valea-ierii.business.site</x:v>
+      </x:c>
+      <x:c r="F111" s="7" t="str"/>
+      <x:c r="G111" s="7" t="str"/>
+      <x:c r="H111" s="7" t="str"/>
+      <x:c r="I111" s="7" t="str">
+        <x:v>https://www.turismvaleaierii.ro/en/cazari-si-servicii</x:v>
+      </x:c>
+      <x:c r="J111" s="13" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="K111" s="7" t="str">
+        <x:v>Cluj / Valea Ierii</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="112" ht="31.5" customHeight="1">
+      <x:c r="A112" s="7" t="str">
+        <x:v>Montagnoli Luxury Cabin</x:v>
+      </x:c>
+      <x:c r="B112" s="7" t="str">
+        <x:v>Cluj</x:v>
+      </x:c>
+      <x:c r="C112" s="7" t="str">
+        <x:v>Valea Ierii, Strada Principală nr. 33A</x:v>
+      </x:c>
+      <x:c r="D112" s="7" t="str">
+        <x:v>+40 787 465 770</x:v>
+      </x:c>
+      <x:c r="E112" s="7" t="str"/>
+      <x:c r="F112" s="7" t="str"/>
+      <x:c r="G112" s="7" t="str"/>
+      <x:c r="H112" s="7" t="str"/>
+      <x:c r="I112" s="7" t="str">
+        <x:v>https://www.turismvaleaierii.ro/en/cazari-si-servicii</x:v>
+      </x:c>
+      <x:c r="J112" s="13" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="K112" s="7" t="str">
+        <x:v>Cluj / Valea Ierii</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="113" ht="31.5" customHeight="1">
+      <x:c r="A113" s="7" t="str">
+        <x:v>Cabana Karla</x:v>
+      </x:c>
+      <x:c r="B113" s="7" t="str">
+        <x:v>Cluj</x:v>
+      </x:c>
+      <x:c r="C113" s="7" t="str">
+        <x:v>Comuna Valea Ierii, sat Cerc</x:v>
+      </x:c>
+      <x:c r="D113" s="7" t="str">
+        <x:v>+40 748 097 785</x:v>
+      </x:c>
+      <x:c r="E113" s="7" t="str"/>
+      <x:c r="F113" s="7" t="str"/>
+      <x:c r="G113" s="7" t="str"/>
+      <x:c r="H113" s="7" t="str"/>
+      <x:c r="I113" s="7" t="str">
+        <x:v>https://www.turismvaleaierii.ro/en/cazari-si-servicii</x:v>
+      </x:c>
+      <x:c r="J113" s="13" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="K113" s="7" t="str">
+        <x:v>Cluj / Valea Ierii-Cerc</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="114" ht="31.5" customHeight="1">
+      <x:c r="A114" s="8" t="str">
+        <x:v>Ama Holiday Home</x:v>
+      </x:c>
+      <x:c r="B114" s="8" t="str">
+        <x:v>Cluj</x:v>
+      </x:c>
+      <x:c r="C114" s="8" t="str">
+        <x:v>Comuna Valea Ierii nr. 95</x:v>
+      </x:c>
+      <x:c r="D114" s="8" t="str">
+        <x:v>+40 745 111 951</x:v>
+      </x:c>
+      <x:c r="E114" s="8" t="str"/>
+      <x:c r="F114" s="8" t="str"/>
+      <x:c r="G114" s="8" t="str"/>
+      <x:c r="H114" s="8" t="str"/>
+      <x:c r="I114" s="8" t="str">
+        <x:v>https://www.turismvaleaierii.ro/en/cazari-si-servicii</x:v>
+      </x:c>
+      <x:c r="J114" s="14" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="K114" s="8" t="str">
+        <x:v>Cluj / Valea Ierii</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
-  <x:conditionalFormatting sqref="J2:J62">
+  <x:conditionalFormatting sqref="J2:J114">
     <x:cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="Outreached"/>
     <x:cfRule type="containsText" dxfId="1" priority="2" operator="containsText" text="Rejected"/>
     <x:cfRule type="containsText" dxfId="2" priority="3" operator="containsText" text="Closed"/>
   </x:conditionalFormatting>
   <x:dataValidations count="1">
-    <x:dataValidation type="list" sqref="J2:J62">
+    <x:dataValidation type="list" sqref="J2:J114">
       <x:formula1>"Pending,Outreached,Rejected,Closed"</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R08e33ef560b143c8"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R538c205da13c4504"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>